<commit_message>
Drafts sheet: mark the 33 deleted rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2g112JF6CCLo8Tg7CRZKC
</commit_message>
<xml_diff>
--- a/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
+++ b/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
@@ -1017,8 +1017,16 @@
           <t>Already live as "Deyga 10% Vitamin C Face Serum 20ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L2" s="16" t="inlineStr"/>
-      <c r="M2" s="13" t="inlineStr"/>
+      <c r="L2" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M2" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N2" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1073,8 +1081,16 @@
           <t>Already live as "Deyga Beautifying Serum 30 ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L3" s="16" t="inlineStr"/>
-      <c r="M3" s="13" t="inlineStr"/>
+      <c r="L3" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N3" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1129,8 +1145,16 @@
           <t>Already live as "Deyga Charcoal Bath Bar 130 g". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L4" s="16" t="inlineStr"/>
-      <c r="M4" s="13" t="inlineStr"/>
+      <c r="L4" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N4" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1297,8 +1321,16 @@
           <t>Already live as "Deyga Rose &amp; Mulethi Skin Brightening Pack 50 g". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L7" s="16" t="inlineStr"/>
-      <c r="M7" s="13" t="inlineStr"/>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N7" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1353,8 +1385,16 @@
           <t>Already live as "Deyga's Under Eye Cream 15 g". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L8" s="16" t="inlineStr"/>
-      <c r="M8" s="13" t="inlineStr"/>
+      <c r="L8" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N8" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1577,8 +1617,16 @@
           <t>Already live as "Jo Milano Unisex Blind Bid P 100 ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L12" s="16" t="inlineStr"/>
-      <c r="M12" s="13" t="inlineStr"/>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M12" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N12" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1857,8 +1905,16 @@
           <t>Already live as "Game Of Spades Moon Unisex Eau De Parfum 100ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L17" s="16" t="inlineStr"/>
-      <c r="M17" s="13" t="inlineStr"/>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N17" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2081,8 +2137,16 @@
           <t>Already live: the Viva La Juicy Rosé listing has a 50ml size (£31.99). Move this draft's stock (2) to that size, then delete.</t>
         </is>
       </c>
-      <c r="L21" s="16" t="inlineStr"/>
-      <c r="M21" s="13" t="inlineStr"/>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M21" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N21" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2137,8 +2201,16 @@
           <t>Already live as "Acqua di Parma Holiday Discovery Set EDP 3x12ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L22" s="16" t="inlineStr"/>
-      <c r="M22" s="13" t="inlineStr"/>
+      <c r="L22" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N22" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2193,8 +2265,16 @@
           <t>Already live as "Giorgio Armani Code Eau de Toilette 125ml Refillable – Men’s Woody Aromatic Fragrance". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L23" s="16" t="inlineStr"/>
-      <c r="M23" s="13" t="inlineStr"/>
+      <c r="L23" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M23" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N23" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -3369,8 +3449,16 @@
           <t>Duplicate draft of "Nusuk Ana Al Awwal Malaki Eau De Parfum for Women" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L44" s="16" t="inlineStr"/>
-      <c r="M44" s="13" t="inlineStr"/>
+      <c r="L44" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M44" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N44" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -3593,8 +3681,16 @@
           <t>Duplicate draft of "Nusuk Ana Al Awwal (Golden) Eau De Parfum for Women" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L48" s="16" t="inlineStr"/>
-      <c r="M48" s="13" t="inlineStr"/>
+      <c r="L48" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M48" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N48" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -3873,8 +3969,16 @@
           <t>Duplicate draft of "Celesto Intense, Eau de Parfum, Riiffs, Unisex, 100 ml" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L53" s="16" t="inlineStr"/>
-      <c r="M53" s="13" t="inlineStr"/>
+      <c r="L53" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M53" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N53" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -4321,8 +4425,16 @@
           <t>Duplicate draft of "LUXURY VERT RiiFFS PARFUM" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L61" s="16" t="inlineStr"/>
-      <c r="M61" s="13" t="inlineStr"/>
+      <c r="L61" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M61" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N61" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -4433,8 +4545,16 @@
           <t>Duplicate draft of "Nusuk Maisan Eau De Parfum for Women | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L63" s="16" t="inlineStr"/>
-      <c r="M63" s="13" t="inlineStr"/>
+      <c r="L63" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M63" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N63" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -4489,8 +4609,16 @@
           <t>Duplicate draft of "Nusuk Malika Red Eau De Parfum for Women | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L64" s="16" t="inlineStr"/>
-      <c r="M64" s="13" t="inlineStr"/>
+      <c r="L64" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M64" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N64" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -4545,8 +4673,16 @@
           <t>Duplicate draft of "Nusuk Malikat Blue Eau De Parfum for Men | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L65" s="16" t="inlineStr"/>
-      <c r="M65" s="13" t="inlineStr"/>
+      <c r="L65" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M65" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N65" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -4657,8 +4793,16 @@
           <t>Duplicate draft of "Nusuk Meshal Arctic Eau De Parfum for Men | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L67" s="16" t="inlineStr"/>
-      <c r="M67" s="13" t="inlineStr"/>
+      <c r="L67" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M67" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N67" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -4881,8 +5025,16 @@
           <t>Duplicate draft of "AGAR NOIR INTENSE" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L71" s="16" t="inlineStr"/>
-      <c r="M71" s="13" t="inlineStr"/>
+      <c r="L71" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M71" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N71" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6169,8 +6321,16 @@
           <t>Duplicate draft of "RiiFFS Exclusive Prive Gold Eau de Parfum 100ml For Unisex | Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L94" s="16" t="inlineStr"/>
-      <c r="M94" s="13" t="inlineStr"/>
+      <c r="L94" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M94" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N94" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6337,8 +6497,16 @@
           <t>Duplicate draft of "Abeer, RiiFFS, Unisex Eau de Parfum, 100 ml" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L97" s="16" t="inlineStr"/>
-      <c r="M97" s="13" t="inlineStr"/>
+      <c r="L97" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M97" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N97" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6617,8 +6785,16 @@
           <t>Duplicate draft of "RiiFFS Aurum Femme Eau de Parfum 100ml For Unisex | Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L102" s="16" t="inlineStr"/>
-      <c r="M102" s="13" t="inlineStr"/>
+      <c r="L102" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M102" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N102" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6673,8 +6849,16 @@
           <t>Duplicate draft of "BELLA ROUGE RiiFFS PARFUM" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L103" s="16" t="inlineStr"/>
-      <c r="M103" s="13" t="inlineStr"/>
+      <c r="L103" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M103" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N103" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6729,8 +6913,16 @@
           <t>Duplicate draft of "BLUE ABSOLUE RiiFFS PARFUM" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L104" s="16" t="inlineStr"/>
-      <c r="M104" s="13" t="inlineStr"/>
+      <c r="L104" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M104" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N104" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6785,8 +6977,16 @@
           <t>Duplicate draft of "CAFE NOIR RiiFFS PARFUM" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L105" s="16" t="inlineStr"/>
-      <c r="M105" s="13" t="inlineStr"/>
+      <c r="L105" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M105" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N105" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6841,8 +7041,16 @@
           <t>Duplicate draft of "Celesto Intense, Eau de Parfum, Riiffs, Unisex, 100 ml" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L106" s="16" t="inlineStr"/>
-      <c r="M106" s="13" t="inlineStr"/>
+      <c r="L106" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M106" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N106" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -7345,8 +7553,16 @@
           <t>Duplicate draft of "RiiFFS Eyad Eau De Parfum 100ml for Men | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L115" s="16" t="inlineStr"/>
-      <c r="M115" s="13" t="inlineStr"/>
+      <c r="L115" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M115" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N115" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -7905,8 +8121,16 @@
           <t>Duplicate draft of "RiiFFS Imperial Rouge Eau De Parfum for Women" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L125" s="16" t="inlineStr"/>
-      <c r="M125" s="13" t="inlineStr"/>
+      <c r="L125" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M125" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N125" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -8129,8 +8353,16 @@
           <t>Duplicate draft of "RiiFFS La Femme Bloom Eau De Parfum for Women" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L129" s="16" t="inlineStr"/>
-      <c r="M129" s="13" t="inlineStr"/>
+      <c r="L129" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M129" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N129" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -8801,8 +9033,16 @@
           <t>Duplicate draft of "RiiFFS Rosa Femme Eau de Parfum 100ml For Unisex | Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L141" s="16" t="inlineStr"/>
-      <c r="M141" s="13" t="inlineStr"/>
+      <c r="L141" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M141" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N141" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -9305,8 +9545,16 @@
           <t>Duplicate draft of "RiiFFS Shanaya Eau de Parfum 100ml For Unisex Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L150" s="16" t="inlineStr"/>
-      <c r="M150" s="13" t="inlineStr"/>
+      <c r="L150" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M150" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N150" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -9361,8 +9609,16 @@
           <t>Duplicate draft of "TANZANITE AMBER" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L151" s="16" t="inlineStr"/>
-      <c r="M151" s="13" t="inlineStr"/>
+      <c r="L151" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M151" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N151" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -9697,8 +9953,16 @@
           <t>Duplicate draft of "Nusuk Sultan Al Arab Eau De Parfum for Men 100ml | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L157" s="16" t="inlineStr"/>
-      <c r="M157" s="13" t="inlineStr"/>
+      <c r="L157" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M157" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N157" s="17" t="inlineStr">
         <is>
           <t>Open</t>

</xml_diff>

<commit_message>
Publish 6 Game of Spades drafts (Jo Milano), hold Vilvah aloe 2-pack
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2g112JF6CCLo8Tg7CRZKC
</commit_message>
<xml_diff>
--- a/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
+++ b/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
@@ -1449,8 +1449,16 @@
           <t>2 in stock. Vendor -&gt; Vilvah, short title, SEO.</t>
         </is>
       </c>
-      <c r="L9" s="16" t="inlineStr"/>
-      <c r="M9" s="13" t="inlineStr"/>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Not sure</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>Held 31 Oct: live Vilvah Aloe Vera Gel already has a 2-pack option (£18.99)</t>
+        </is>
+      </c>
       <c r="N9" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1561,8 +1569,16 @@
           <t>Not on the site yet and 14 in stock. Needs vendor Jo Milano, short title, SEO title/description.</t>
         </is>
       </c>
-      <c r="L11" s="16" t="inlineStr"/>
-      <c r="M11" s="13" t="inlineStr"/>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Finish &amp; publish</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>Published 31 Oct 2026 (vendor Jo Milano, SEO, alt text)</t>
+        </is>
+      </c>
       <c r="N11" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1681,8 +1697,16 @@
           <t>Not on the site yet and 23 in stock. Needs vendor Jo Milano, short title, SEO title/description.</t>
         </is>
       </c>
-      <c r="L13" s="16" t="inlineStr"/>
-      <c r="M13" s="13" t="inlineStr"/>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Finish &amp; publish</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t>Published 31 Oct 2026 (vendor Jo Milano, SEO, alt text)</t>
+        </is>
+      </c>
       <c r="N13" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1737,8 +1761,16 @@
           <t>Not on the site yet and 5 in stock. Needs vendor Jo Milano, short title, SEO title/description.</t>
         </is>
       </c>
-      <c r="L14" s="16" t="inlineStr"/>
-      <c r="M14" s="13" t="inlineStr"/>
+      <c r="L14" s="16" t="inlineStr">
+        <is>
+          <t>Finish &amp; publish</t>
+        </is>
+      </c>
+      <c r="M14" s="13" t="inlineStr">
+        <is>
+          <t>Published 31 Oct 2026 (vendor Jo Milano, SEO, alt text)</t>
+        </is>
+      </c>
       <c r="N14" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1793,8 +1825,16 @@
           <t>Not on the site yet and 15 in stock. Needs vendor Jo Milano, short title, SEO title/description.</t>
         </is>
       </c>
-      <c r="L15" s="16" t="inlineStr"/>
-      <c r="M15" s="13" t="inlineStr"/>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Finish &amp; publish</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>Published 31 Oct 2026 (vendor Jo Milano, SEO, alt text)</t>
+        </is>
+      </c>
       <c r="N15" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1849,8 +1889,16 @@
           <t>Not on the site yet and 25 in stock. Needs vendor Jo Milano, short title, SEO title/description.</t>
         </is>
       </c>
-      <c r="L16" s="16" t="inlineStr"/>
-      <c r="M16" s="13" t="inlineStr"/>
+      <c r="L16" s="16" t="inlineStr">
+        <is>
+          <t>Finish &amp; publish</t>
+        </is>
+      </c>
+      <c r="M16" s="13" t="inlineStr">
+        <is>
+          <t>Published 31 Oct 2026 (vendor Jo Milano, SEO, alt text)</t>
+        </is>
+      </c>
       <c r="N16" s="17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1969,8 +2017,16 @@
           <t>Not on the site yet and 7 in stock. Needs vendor Jo Milano, short title, SEO title/description.</t>
         </is>
       </c>
-      <c r="L18" s="16" t="inlineStr"/>
-      <c r="M18" s="13" t="inlineStr"/>
+      <c r="L18" s="16" t="inlineStr">
+        <is>
+          <t>Finish &amp; publish</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr">
+        <is>
+          <t>Published 31 Oct 2026 (vendor Jo Milano, SEO, alt text)</t>
+        </is>
+      </c>
       <c r="N18" s="17" t="inlineStr">
         <is>
           <t>Open</t>

</xml_diff>

<commit_message>
Delete Vilvah aloe 2-pack draft, move its stock to the live 2-pack option
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2g112JF6CCLo8Tg7CRZKC
</commit_message>
<xml_diff>
--- a/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
+++ b/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
@@ -1451,12 +1451,12 @@
       </c>
       <c r="L9" s="16" t="inlineStr">
         <is>
-          <t>Not sure</t>
+          <t>Delete</t>
         </is>
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>Held 31 Oct: live Vilvah Aloe Vera Gel already has a 2-pack option (£18.99)</t>
+          <t>Deleted 31 Oct 2026; its 2 units moved to the live Aloe Vera Gel "2" option (1 → 3)</t>
         </is>
       </c>
       <c r="N9" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Delete Vilvah Melt-in-Milk Sunscreen draft (backup kept)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2g112JF6CCLo8Tg7CRZKC
</commit_message>
<xml_diff>
--- a/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
+++ b/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
@@ -1513,8 +1513,16 @@
           <t>0 in stock. Vilvah now sells Skin Finish Sunscreen (live). Delete unless you will restock Melt-in-Milk.</t>
         </is>
       </c>
-      <c r="L10" s="16" t="inlineStr"/>
-      <c r="M10" s="13" t="inlineStr"/>
+      <c r="L10" s="16" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>Deleted 31 Oct 2026 (backup kept)</t>
+        </is>
+      </c>
       <c r="N10" s="17" t="inlineStr">
         <is>
           <t>Open</t>

</xml_diff>

<commit_message>
Restore the 35 deleted drafts from backups (no photos), reverse aloe stock move
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2g112JF6CCLo8Tg7CRZKC
</commit_message>
<xml_diff>
--- a/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
+++ b/docs/Swansura_Old_Draft_Products_2026-10-31.xlsx
@@ -1017,14 +1017,10 @@
           <t>Already live as "Deyga 10% Vitamin C Face Serum 20ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L2" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L2" s="16" t="n"/>
       <c r="M2" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N2" s="17" t="inlineStr">
@@ -1081,14 +1077,10 @@
           <t>Already live as "Deyga Beautifying Serum 30 ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L3" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L3" s="16" t="n"/>
       <c r="M3" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N3" s="17" t="inlineStr">
@@ -1145,14 +1137,10 @@
           <t>Already live as "Deyga Charcoal Bath Bar 130 g". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L4" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L4" s="16" t="n"/>
       <c r="M4" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N4" s="17" t="inlineStr">
@@ -1321,14 +1309,10 @@
           <t>Already live as "Deyga Rose &amp; Mulethi Skin Brightening Pack 50 g". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L7" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L7" s="16" t="n"/>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N7" s="17" t="inlineStr">
@@ -1385,14 +1369,10 @@
           <t>Already live as "Deyga's Under Eye Cream 15 g". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L8" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L8" s="16" t="n"/>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N8" s="17" t="inlineStr">
@@ -1449,14 +1429,10 @@
           <t>2 in stock. Vendor -&gt; Vilvah, short title, SEO.</t>
         </is>
       </c>
-      <c r="L9" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L9" s="16" t="n"/>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026; its 2 units moved to the live Aloe Vera Gel "2" option (1 → 3)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N9" s="17" t="inlineStr">
@@ -1513,14 +1489,10 @@
           <t>0 in stock. Vilvah now sells Skin Finish Sunscreen (live). Delete unless you will restock Melt-in-Milk.</t>
         </is>
       </c>
-      <c r="L10" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L10" s="16" t="n"/>
       <c r="M10" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N10" s="17" t="inlineStr">
@@ -1641,14 +1613,10 @@
           <t>Already live as "Jo Milano Unisex Blind Bid P 100 ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L12" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L12" s="16" t="n"/>
       <c r="M12" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N12" s="17" t="inlineStr">
@@ -1961,14 +1929,10 @@
           <t>Already live as "Game Of Spades Moon Unisex Eau De Parfum 100ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L17" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L17" s="16" t="n"/>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N17" s="17" t="inlineStr">
@@ -2201,14 +2165,10 @@
           <t>Already live: the Viva La Juicy Rosé listing has a 50ml size (£31.99). Move this draft's stock (2) to that size, then delete.</t>
         </is>
       </c>
-      <c r="L21" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L21" s="16" t="n"/>
       <c r="M21" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N21" s="17" t="inlineStr">
@@ -2265,14 +2225,10 @@
           <t>Already live as "Acqua di Parma Holiday Discovery Set EDP 3x12ml". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L22" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L22" s="16" t="n"/>
       <c r="M22" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N22" s="17" t="inlineStr">
@@ -2329,14 +2285,10 @@
           <t>Already live as "Giorgio Armani Code Eau de Toilette 125ml Refillable – Men’s Woody Aromatic Fragrance". This draft is a copy.</t>
         </is>
       </c>
-      <c r="L23" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L23" s="16" t="n"/>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N23" s="17" t="inlineStr">
@@ -3513,14 +3465,10 @@
           <t>Duplicate draft of "Nusuk Ana Al Awwal Malaki Eau De Parfum for Women" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L44" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L44" s="16" t="n"/>
       <c r="M44" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N44" s="17" t="inlineStr">
@@ -3745,14 +3693,10 @@
           <t>Duplicate draft of "Nusuk Ana Al Awwal (Golden) Eau De Parfum for Women" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L48" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L48" s="16" t="n"/>
       <c r="M48" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N48" s="17" t="inlineStr">
@@ -4033,14 +3977,10 @@
           <t>Duplicate draft of "Celesto Intense, Eau de Parfum, Riiffs, Unisex, 100 ml" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L53" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L53" s="16" t="n"/>
       <c r="M53" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N53" s="17" t="inlineStr">
@@ -4489,14 +4429,10 @@
           <t>Duplicate draft of "LUXURY VERT RiiFFS PARFUM" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L61" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L61" s="16" t="n"/>
       <c r="M61" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N61" s="17" t="inlineStr">
@@ -4609,14 +4545,10 @@
           <t>Duplicate draft of "Nusuk Maisan Eau De Parfum for Women | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L63" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L63" s="16" t="n"/>
       <c r="M63" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N63" s="17" t="inlineStr">
@@ -4673,14 +4605,10 @@
           <t>Duplicate draft of "Nusuk Malika Red Eau De Parfum for Women | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L64" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L64" s="16" t="n"/>
       <c r="M64" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N64" s="17" t="inlineStr">
@@ -4737,14 +4665,10 @@
           <t>Duplicate draft of "Nusuk Malikat Blue Eau De Parfum for Men | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L65" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L65" s="16" t="n"/>
       <c r="M65" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N65" s="17" t="inlineStr">
@@ -4857,14 +4781,10 @@
           <t>Duplicate draft of "Nusuk Meshal Arctic Eau De Parfum for Men | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L67" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L67" s="16" t="n"/>
       <c r="M67" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N67" s="17" t="inlineStr">
@@ -5089,14 +5009,10 @@
           <t>Duplicate draft of "AGAR NOIR INTENSE" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L71" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L71" s="16" t="n"/>
       <c r="M71" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N71" s="17" t="inlineStr">
@@ -6385,14 +6301,10 @@
           <t>Duplicate draft of "RiiFFS Exclusive Prive Gold Eau de Parfum 100ml For Unisex | Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L94" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L94" s="16" t="n"/>
       <c r="M94" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N94" s="17" t="inlineStr">
@@ -6561,14 +6473,10 @@
           <t>Duplicate draft of "Abeer, RiiFFS, Unisex Eau de Parfum, 100 ml" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L97" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L97" s="16" t="n"/>
       <c r="M97" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N97" s="17" t="inlineStr">
@@ -6849,14 +6757,10 @@
           <t>Duplicate draft of "RiiFFS Aurum Femme Eau de Parfum 100ml For Unisex | Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L102" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L102" s="16" t="n"/>
       <c r="M102" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N102" s="17" t="inlineStr">
@@ -6913,14 +6817,10 @@
           <t>Duplicate draft of "BELLA ROUGE RiiFFS PARFUM" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L103" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L103" s="16" t="n"/>
       <c r="M103" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N103" s="17" t="inlineStr">
@@ -6977,14 +6877,10 @@
           <t>Duplicate draft of "BLUE ABSOLUE RiiFFS PARFUM" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L104" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L104" s="16" t="n"/>
       <c r="M104" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N104" s="17" t="inlineStr">
@@ -7041,14 +6937,10 @@
           <t>Duplicate draft of "CAFE NOIR RiiFFS PARFUM" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L105" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L105" s="16" t="n"/>
       <c r="M105" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N105" s="17" t="inlineStr">
@@ -7105,14 +6997,10 @@
           <t>Duplicate draft of "Celesto Intense, Eau de Parfum, Riiffs, Unisex, 100 ml" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L106" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L106" s="16" t="n"/>
       <c r="M106" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N106" s="17" t="inlineStr">
@@ -7617,14 +7505,10 @@
           <t>Duplicate draft of "RiiFFS Eyad Eau De Parfum 100ml for Men | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L115" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L115" s="16" t="n"/>
       <c r="M115" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N115" s="17" t="inlineStr">
@@ -8185,14 +8069,10 @@
           <t>Duplicate draft of "RiiFFS Imperial Rouge Eau De Parfum for Women" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L125" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L125" s="16" t="n"/>
       <c r="M125" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N125" s="17" t="inlineStr">
@@ -8417,14 +8297,10 @@
           <t>Duplicate draft of "RiiFFS La Femme Bloom Eau De Parfum for Women" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L129" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L129" s="16" t="n"/>
       <c r="M129" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N129" s="17" t="inlineStr">
@@ -9097,14 +8973,10 @@
           <t>Duplicate draft of "RiiFFS Rosa Femme Eau de Parfum 100ml For Unisex | Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L141" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L141" s="16" t="n"/>
       <c r="M141" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N141" s="17" t="inlineStr">
@@ -9609,14 +9481,10 @@
           <t>Duplicate draft of "RiiFFS Shanaya Eau de Parfum 100ml For Unisex Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L150" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L150" s="16" t="n"/>
       <c r="M150" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N150" s="17" t="inlineStr">
@@ -9673,14 +9541,10 @@
           <t>Duplicate draft of "TANZANITE AMBER" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L151" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L151" s="16" t="n"/>
       <c r="M151" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N151" s="17" t="inlineStr">
@@ -10017,14 +9881,10 @@
           <t>Duplicate draft of "Nusuk Sultan Al Arab Eau De Parfum for Men 100ml | Long-Lasting Luxury Fragrance" (same perfume listed twice).</t>
         </is>
       </c>
-      <c r="L157" s="16" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
+      <c r="L157" s="16" t="n"/>
       <c r="M157" s="13" t="inlineStr">
         <is>
-          <t>Deleted 31 Oct 2026 (backup kept)</t>
+          <t>Deleted then restored 31 Oct 2026 as a draft (same text, price, SKU, stock); photos could not be restored</t>
         </is>
       </c>
       <c r="N157" s="17" t="inlineStr">

</xml_diff>